<commit_message>
Updated the CC_Method_Analysis_v_0_1.py script to remove the document.save() function call in the linearityreport function, as it was causing issues with saving the document, different names that the user may provide. Saving the linearity report is now handled outside of the CC module. Also removed the linearity interval with error, as it did not make sense mathematically. It is not defined by stretching the extreme ends of your assay by their confidence intervals.
</commit_message>
<xml_diff>
--- a/Liprotein_a.xlsx
+++ b/Liprotein_a.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityhealthnetwork-my.sharepoint.com/personal/rajeevan_selvaratnam_uhn_ca/Documents/R Scripts/My Python Modules for CC Method Comp/PyME/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{CC3D98EC-1BA9-4303-A39B-7D4FB561D130}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44F414BE-9B9D-4074-A91E-EFFC29D40EDB}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{CC3D98EC-1BA9-4303-A39B-7D4FB561D130}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17C440A2-4FF5-4AF8-B8E0-4C6B458C78C5}"/>
   <bookViews>
-    <workbookView xWindow="-2750" yWindow="-21600" windowWidth="19380" windowHeight="20970" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="24721" windowHeight="15826" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Method Comparison" sheetId="1" r:id="rId1"/>
@@ -431,9 +431,6 @@
     <t>If available, provide the expected mean and/or range from the manufacturer</t>
   </si>
   <si>
-    <t>Expected Mean</t>
-  </si>
-  <si>
     <t>Expected Range</t>
   </si>
   <si>
@@ -485,13 +482,16 @@
   <si>
     <t>Level 10</t>
   </si>
+  <si>
+    <t>Expected Result</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="#,##0.000"/>
+    <numFmt numFmtId="164" formatCode="#,##0.000"/>
   </numFmts>
   <fonts count="37" x14ac:knownFonts="1">
     <font>
@@ -1681,36 +1681,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="28" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="4"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="4" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1748,15 +1718,6 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="4" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="30" fillId="2" borderId="17" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="31" fillId="0" borderId="23" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="24" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="1" xfId="4" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1772,25 +1733,7 @@
     <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="4" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="30" fillId="2" borderId="25" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="31" fillId="0" borderId="3" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="27" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="30" fillId="2" borderId="20" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="31" fillId="0" borderId="28" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="29" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="4" applyFont="1"/>
@@ -1801,56 +1744,11 @@
     <xf numFmtId="3" fontId="25" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="33" fillId="2" borderId="30" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="33" fillId="2" borderId="31" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="33" fillId="2" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="33" fillId="2" borderId="20" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="33" fillId="2" borderId="21" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="33" fillId="2" borderId="22" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="26" fillId="10" borderId="33" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="26" fillId="10" borderId="34" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="26" fillId="10" borderId="35" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="26" fillId="10" borderId="36" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="26" fillId="10" borderId="1" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="26" fillId="10" borderId="37" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="26" fillId="10" borderId="38" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="26" fillId="10" borderId="39" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="26" fillId="10" borderId="40" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="11" borderId="1" xfId="3" applyBorder="1"/>
     <xf numFmtId="3" fontId="25" fillId="11" borderId="1" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1860,19 +1758,121 @@
     <xf numFmtId="3" fontId="26" fillId="10" borderId="1" xfId="5" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="29" fillId="2" borderId="18" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="29" fillId="2" borderId="18" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="29" fillId="2" borderId="21" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="29" fillId="2" borderId="21" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="29" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="30" fillId="2" borderId="2" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="2" borderId="2" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="1" xfId="4" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="1" xfId="4" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="33" fillId="2" borderId="20" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="33" fillId="2" borderId="21" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="33" fillId="2" borderId="22" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="26" fillId="10" borderId="33" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="26" fillId="10" borderId="34" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="26" fillId="10" borderId="35" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="26" fillId="10" borderId="36" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="26" fillId="10" borderId="1" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="26" fillId="10" borderId="37" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="26" fillId="10" borderId="38" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="26" fillId="10" borderId="39" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="26" fillId="10" borderId="40" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="28" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="30" fillId="2" borderId="17" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="31" fillId="0" borderId="23" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="24" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="30" fillId="2" borderId="25" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="31" fillId="0" borderId="3" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="27" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="30" fillId="2" borderId="20" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="31" fillId="0" borderId="28" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="29" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="33" fillId="2" borderId="30" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="33" fillId="2" borderId="31" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="33" fillId="2" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="20% - Accent1" xfId="3" builtinId="30"/>
@@ -1884,7 +1884,7 @@
   </cellStyles>
   <dxfs count="1">
     <dxf>
-      <numFmt numFmtId="166" formatCode="#,##0.000"/>
+      <numFmt numFmtId="164" formatCode="#,##0.000"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1902,6 +1902,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1929,7 +1933,7 @@
     <tableColumn id="2" xr3:uid="{22C03DAC-E0AC-4097-ACE8-D5161FC2B6E3}" name="Replicate"/>
     <tableColumn id="3" xr3:uid="{E082759A-6253-4B2A-B1C9-2F7C040B5290}" name="Measured Result"/>
     <tableColumn id="4" xr3:uid="{58B09B39-044F-411E-96B8-127F274870BE}" name="Average" dataDxfId="0"/>
-    <tableColumn id="5" xr3:uid="{268B30F7-6AC1-4A9B-8B41-E7B2632FDCEE}" name="Expected Mean"/>
+    <tableColumn id="5" xr3:uid="{268B30F7-6AC1-4A9B-8B41-E7B2632FDCEE}" name="Expected Result"/>
     <tableColumn id="6" xr3:uid="{CA8FE3C4-7DE9-456C-8635-FE1C15E492C8}" name="Expected Range"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2298,13 +2302,13 @@
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="149" t="s">
+      <c r="B5" s="203" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="146"/>
-      <c r="D5" s="146"/>
-      <c r="E5" s="146"/>
-      <c r="F5" s="147"/>
+      <c r="C5" s="204"/>
+      <c r="D5" s="204"/>
+      <c r="E5" s="204"/>
+      <c r="F5" s="205"/>
     </row>
     <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B6" s="5"/>
@@ -2439,10 +2443,10 @@
       <c r="A21" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="150"/>
-      <c r="C21" s="146"/>
-      <c r="D21" s="146"/>
-      <c r="E21" s="151"/>
+      <c r="B21" s="206"/>
+      <c r="C21" s="204"/>
+      <c r="D21" s="204"/>
+      <c r="E21" s="207"/>
     </row>
     <row r="22" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="91" t="s">
@@ -3729,15 +3733,15 @@
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="149" t="str">
+      <c r="B5" s="203" t="str">
         <f>'Method Comparison'!B5:F5</f>
         <v>This method serves to bringing in-house BNP testing for heart failure assessments</v>
       </c>
-      <c r="C5" s="146"/>
-      <c r="D5" s="146"/>
-      <c r="E5" s="152"/>
-      <c r="F5" s="146"/>
-      <c r="G5" s="151"/>
+      <c r="C5" s="204"/>
+      <c r="D5" s="204"/>
+      <c r="E5" s="208"/>
+      <c r="F5" s="204"/>
+      <c r="G5" s="207"/>
       <c r="H5" s="53"/>
     </row>
     <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -10104,177 +10108,221 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:K59"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="33" style="154" customWidth="1"/>
-    <col min="2" max="2" width="9.796875" style="185" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.06640625" style="184" customWidth="1"/>
-    <col min="4" max="4" width="13.59765625" style="211" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.59765625" style="184" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.33203125" style="154" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.06640625" style="154"/>
+    <col min="1" max="1" width="33" style="144" customWidth="1"/>
+    <col min="2" max="2" width="9.796875" style="166" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.06640625" style="165" customWidth="1"/>
+    <col min="4" max="4" width="13.59765625" style="177" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.59765625" style="165" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.33203125" style="144" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.06640625" style="144"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="153" t="s">
+    <row r="1" spans="1:12" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="190" t="s">
         <v>124</v>
       </c>
-      <c r="B1" s="153"/>
-      <c r="C1" s="153"/>
-      <c r="D1" s="153"/>
-      <c r="E1" s="153"/>
-      <c r="F1" s="153"/>
-      <c r="G1" s="153"/>
-      <c r="H1" s="153"/>
-      <c r="I1" s="153"/>
-      <c r="J1" s="153"/>
-      <c r="K1" s="153"/>
-    </row>
-    <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="155" t="s">
+      <c r="B1" s="190"/>
+      <c r="C1" s="190"/>
+      <c r="D1" s="190"/>
+      <c r="E1" s="190"/>
+      <c r="F1" s="190"/>
+      <c r="G1" s="190"/>
+      <c r="H1" s="190"/>
+      <c r="I1" s="190"/>
+      <c r="J1" s="190"/>
+      <c r="K1" s="190"/>
+    </row>
+    <row r="2" spans="1:12" ht="18.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="145" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="156" t="s">
-        <v>135</v>
-      </c>
-      <c r="C2" s="157"/>
-      <c r="D2" s="207"/>
-      <c r="E2" s="158"/>
-      <c r="F2" s="159"/>
-    </row>
-    <row r="3" spans="1:11" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A3" s="160" t="s">
+      <c r="B2" s="146" t="s">
+        <v>134</v>
+      </c>
+      <c r="C2" s="147"/>
+      <c r="D2" s="173"/>
+      <c r="E2" s="148"/>
+      <c r="F2" s="149"/>
+      <c r="G2" s="181" t="s">
+        <v>133</v>
+      </c>
+      <c r="H2" s="182"/>
+      <c r="I2" s="182"/>
+      <c r="J2" s="182"/>
+      <c r="K2" s="182"/>
+      <c r="L2" s="183"/>
+    </row>
+    <row r="3" spans="1:12" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A3" s="150" t="s">
         <v>97</v>
       </c>
-      <c r="B3" s="161" t="s">
+      <c r="B3" s="151" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="162"/>
-      <c r="D3" s="208"/>
-      <c r="E3" s="163"/>
-      <c r="F3" s="164"/>
-    </row>
-    <row r="4" spans="1:11" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A4" s="160"/>
-      <c r="B4" s="165"/>
-      <c r="C4" s="165"/>
-      <c r="D4" s="209"/>
-      <c r="E4" s="165"/>
-      <c r="F4" s="166"/>
-    </row>
-    <row r="5" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="166" t="s">
+      <c r="C3" s="152"/>
+      <c r="D3" s="174"/>
+      <c r="E3" s="153"/>
+      <c r="F3" s="154"/>
+      <c r="G3" s="184"/>
+      <c r="H3" s="185"/>
+      <c r="I3" s="185"/>
+      <c r="J3" s="185"/>
+      <c r="K3" s="185"/>
+      <c r="L3" s="186"/>
+    </row>
+    <row r="4" spans="1:12" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A4" s="150"/>
+      <c r="B4" s="155"/>
+      <c r="C4" s="155"/>
+      <c r="D4" s="175"/>
+      <c r="E4" s="155"/>
+      <c r="F4" s="156"/>
+      <c r="G4" s="184"/>
+      <c r="H4" s="185"/>
+      <c r="I4" s="185"/>
+      <c r="J4" s="185"/>
+      <c r="K4" s="185"/>
+      <c r="L4" s="186"/>
+    </row>
+    <row r="5" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A5" s="156" t="s">
         <v>98</v>
       </c>
-      <c r="B5" s="167"/>
-      <c r="C5" s="168"/>
-      <c r="D5" s="168"/>
-      <c r="E5" s="168"/>
-      <c r="F5" s="169"/>
-    </row>
-    <row r="6" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="170" t="s">
+      <c r="B5" s="191"/>
+      <c r="C5" s="192"/>
+      <c r="D5" s="192"/>
+      <c r="E5" s="192"/>
+      <c r="F5" s="193"/>
+      <c r="G5" s="184"/>
+      <c r="H5" s="185"/>
+      <c r="I5" s="185"/>
+      <c r="J5" s="185"/>
+      <c r="K5" s="185"/>
+      <c r="L5" s="186"/>
+    </row>
+    <row r="6" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="157" t="s">
         <v>99</v>
       </c>
-      <c r="B6" s="171"/>
-      <c r="C6" s="172"/>
-      <c r="D6" s="210"/>
-      <c r="E6" s="172"/>
-      <c r="F6" s="173"/>
-    </row>
-    <row r="7" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="174" t="s">
+      <c r="B6" s="158"/>
+      <c r="C6" s="159"/>
+      <c r="D6" s="176"/>
+      <c r="E6" s="159"/>
+      <c r="F6" s="160"/>
+      <c r="G6" s="184"/>
+      <c r="H6" s="185"/>
+      <c r="I6" s="185"/>
+      <c r="J6" s="185"/>
+      <c r="K6" s="185"/>
+      <c r="L6" s="186"/>
+    </row>
+    <row r="7" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="161" t="s">
         <v>100</v>
       </c>
-      <c r="B7" s="175"/>
-      <c r="C7" s="176"/>
-      <c r="D7" s="176"/>
-      <c r="E7" s="176"/>
-      <c r="F7" s="177"/>
-    </row>
-    <row r="8" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="174" t="s">
+      <c r="B7" s="194"/>
+      <c r="C7" s="195"/>
+      <c r="D7" s="195"/>
+      <c r="E7" s="195"/>
+      <c r="F7" s="196"/>
+      <c r="G7" s="184"/>
+      <c r="H7" s="185"/>
+      <c r="I7" s="185"/>
+      <c r="J7" s="185"/>
+      <c r="K7" s="185"/>
+      <c r="L7" s="186"/>
+    </row>
+    <row r="8" spans="1:12" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A8" s="161" t="s">
         <v>101</v>
       </c>
-      <c r="B8" s="175"/>
-      <c r="C8" s="176"/>
-      <c r="D8" s="176"/>
-      <c r="E8" s="176"/>
-      <c r="F8" s="177"/>
-    </row>
-    <row r="9" spans="1:11" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A9" s="178" t="s">
+      <c r="B8" s="194"/>
+      <c r="C8" s="195"/>
+      <c r="D8" s="195"/>
+      <c r="E8" s="195"/>
+      <c r="F8" s="196"/>
+      <c r="G8" s="187"/>
+      <c r="H8" s="188"/>
+      <c r="I8" s="188"/>
+      <c r="J8" s="188"/>
+      <c r="K8" s="188"/>
+      <c r="L8" s="189"/>
+    </row>
+    <row r="9" spans="1:12" ht="18.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A9" s="162" t="s">
         <v>102</v>
       </c>
-      <c r="B9" s="179"/>
-      <c r="C9" s="180"/>
-      <c r="D9" s="180"/>
-      <c r="E9" s="180"/>
-      <c r="F9" s="181"/>
-    </row>
-    <row r="10" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="182" t="s">
+      <c r="B9" s="197"/>
+      <c r="C9" s="198"/>
+      <c r="D9" s="198"/>
+      <c r="E9" s="198"/>
+      <c r="F9" s="199"/>
+    </row>
+    <row r="10" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A10" s="163" t="s">
         <v>125</v>
       </c>
-      <c r="B10" s="183" t="s">
+      <c r="B10" s="164" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="12" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="182" t="s">
+    <row r="11" spans="1:12" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="12" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A12" s="163" t="s">
         <v>127</v>
       </c>
-      <c r="B12" s="186" t="s">
+      <c r="B12" s="200" t="s">
         <v>128</v>
       </c>
-      <c r="C12" s="187"/>
-      <c r="D12" s="187"/>
-      <c r="E12" s="187"/>
-      <c r="F12" s="188"/>
-    </row>
-    <row r="13" spans="1:11" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B13" s="189" t="s">
+      <c r="C12" s="201"/>
+      <c r="D12" s="201"/>
+      <c r="E12" s="201"/>
+      <c r="F12" s="202"/>
+    </row>
+    <row r="13" spans="1:12" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B13" s="178" t="s">
         <v>129</v>
       </c>
-      <c r="C13" s="190"/>
-      <c r="D13" s="190"/>
-      <c r="E13" s="190"/>
-      <c r="F13" s="191"/>
-    </row>
-    <row r="14" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="15" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="154" t="s">
+      <c r="C13" s="179"/>
+      <c r="D13" s="179"/>
+      <c r="E13" s="179"/>
+      <c r="F13" s="180"/>
+    </row>
+    <row r="14" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="15" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="144" t="s">
         <v>103</v>
       </c>
-      <c r="B15" s="185" t="s">
+      <c r="B15" s="166" t="s">
         <v>70</v>
       </c>
-      <c r="C15" s="184" t="s">
+      <c r="C15" s="165" t="s">
         <v>104</v>
       </c>
-      <c r="D15" s="211" t="s">
+      <c r="D15" s="177" t="s">
         <v>105</v>
       </c>
-      <c r="E15" s="184" t="s">
+      <c r="E15" s="165" t="s">
+        <v>140</v>
+      </c>
+      <c r="F15" s="144" t="s">
         <v>130</v>
       </c>
-      <c r="F15" s="154" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="203" t="s">
+    </row>
+    <row r="16" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="169" t="s">
         <v>66</v>
       </c>
-      <c r="B16" s="204">
+      <c r="B16" s="170">
         <v>1</v>
       </c>
       <c r="C16">
         <v>325.7</v>
       </c>
-      <c r="D16" s="193">
+      <c r="D16" s="168">
         <f>AVERAGE(C16:C18)</f>
         <v>322.35000000000002</v>
       </c>
@@ -10283,10 +10331,10 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="203" t="s">
+      <c r="A17" s="169" t="s">
         <v>66</v>
       </c>
-      <c r="B17" s="204">
+      <c r="B17" s="170">
         <v>2</v>
       </c>
       <c r="C17">
@@ -10294,24 +10342,24 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="203" t="s">
+      <c r="A18" s="169" t="s">
         <v>66</v>
       </c>
-      <c r="B18" s="204">
+      <c r="B18" s="170">
         <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="205" t="s">
-        <v>132</v>
-      </c>
-      <c r="B19" s="206">
+      <c r="A19" s="171" t="s">
+        <v>131</v>
+      </c>
+      <c r="B19" s="172">
         <v>1</v>
       </c>
       <c r="C19">
         <v>273.5</v>
       </c>
-      <c r="D19" s="193">
+      <c r="D19" s="168">
         <f>AVERAGE(C19:C20)</f>
         <v>272.8</v>
       </c>
@@ -10320,10 +10368,10 @@
       </c>
     </row>
     <row r="20" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="205" t="s">
-        <v>132</v>
-      </c>
-      <c r="B20" s="206">
+      <c r="A20" s="171" t="s">
+        <v>131</v>
+      </c>
+      <c r="B20" s="172">
         <v>2</v>
       </c>
       <c r="C20">
@@ -10331,25 +10379,25 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="205" t="s">
-        <v>132</v>
-      </c>
-      <c r="B21" s="206">
+      <c r="A21" s="171" t="s">
+        <v>131</v>
+      </c>
+      <c r="B21" s="172">
         <v>3</v>
       </c>
-      <c r="C21" s="192"/>
+      <c r="C21" s="167"/>
     </row>
     <row r="22" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="203" t="s">
+      <c r="A22" s="169" t="s">
         <v>67</v>
       </c>
-      <c r="B22" s="204">
+      <c r="B22" s="170">
         <v>1</v>
       </c>
       <c r="C22">
         <v>196.8</v>
       </c>
-      <c r="D22" s="193">
+      <c r="D22" s="168">
         <f>AVERAGE(C22:C24)</f>
         <v>196.60000000000002</v>
       </c>
@@ -10358,38 +10406,38 @@
       </c>
     </row>
     <row r="23" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="203" t="s">
+      <c r="A23" s="169" t="s">
         <v>67</v>
       </c>
-      <c r="B23" s="204">
+      <c r="B23" s="170">
         <v>2</v>
       </c>
       <c r="C23">
         <v>196.4</v>
       </c>
-      <c r="D23" s="193"/>
+      <c r="D23" s="168"/>
     </row>
     <row r="24" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A24" s="203" t="s">
+      <c r="A24" s="169" t="s">
         <v>67</v>
       </c>
-      <c r="B24" s="204">
+      <c r="B24" s="170">
         <v>3</v>
       </c>
-      <c r="C24" s="192"/>
-      <c r="D24" s="193"/>
+      <c r="C24" s="167"/>
+      <c r="D24" s="168"/>
     </row>
     <row r="25" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="205" t="s">
+      <c r="A25" s="171" t="s">
         <v>68</v>
       </c>
-      <c r="B25" s="206">
+      <c r="B25" s="172">
         <v>1</v>
       </c>
       <c r="C25">
         <v>169.9</v>
       </c>
-      <c r="D25" s="193">
+      <c r="D25" s="168">
         <f>AVERAGE(C25:C27)</f>
         <v>169.5</v>
       </c>
@@ -10398,32 +10446,32 @@
       </c>
     </row>
     <row r="26" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A26" s="205" t="s">
+      <c r="A26" s="171" t="s">
         <v>68</v>
       </c>
-      <c r="B26" s="206">
+      <c r="B26" s="172">
         <v>2</v>
       </c>
       <c r="C26">
         <v>169.1</v>
       </c>
-      <c r="D26" s="193"/>
+      <c r="D26" s="168"/>
     </row>
     <row r="27" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="205" t="s">
+      <c r="A27" s="171" t="s">
         <v>68</v>
       </c>
-      <c r="B27" s="206">
+      <c r="B27" s="172">
         <v>3</v>
       </c>
-      <c r="C27" s="192"/>
-      <c r="D27" s="193"/>
+      <c r="C27" s="167"/>
+      <c r="D27" s="168"/>
     </row>
     <row r="28" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A28" s="203" t="s">
-        <v>133</v>
-      </c>
-      <c r="B28" s="204">
+      <c r="A28" s="169" t="s">
+        <v>132</v>
+      </c>
+      <c r="B28" s="170">
         <v>1</v>
       </c>
       <c r="C28">
@@ -10437,10 +10485,10 @@
       </c>
     </row>
     <row r="29" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="203" t="s">
-        <v>133</v>
-      </c>
-      <c r="B29" s="204">
+      <c r="A29" s="169" t="s">
+        <v>132</v>
+      </c>
+      <c r="B29" s="170">
         <v>2</v>
       </c>
       <c r="C29">
@@ -10449,26 +10497,26 @@
       <c r="D29"/>
     </row>
     <row r="30" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="203" t="s">
-        <v>133</v>
-      </c>
-      <c r="B30" s="204">
+      <c r="A30" s="169" t="s">
+        <v>132</v>
+      </c>
+      <c r="B30" s="170">
         <v>3</v>
       </c>
-      <c r="C30" s="192"/>
-      <c r="D30" s="193"/>
+      <c r="C30" s="167"/>
+      <c r="D30" s="168"/>
     </row>
     <row r="31" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="205" t="s">
-        <v>136</v>
-      </c>
-      <c r="B31" s="206">
+      <c r="A31" s="171" t="s">
+        <v>135</v>
+      </c>
+      <c r="B31" s="172">
         <v>1</v>
       </c>
       <c r="C31">
         <v>116.1</v>
       </c>
-      <c r="D31" s="193">
+      <c r="D31" s="168">
         <f>AVERAGE(C31:C33)</f>
         <v>115.6</v>
       </c>
@@ -10477,38 +10525,38 @@
       </c>
     </row>
     <row r="32" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="205" t="s">
-        <v>136</v>
-      </c>
-      <c r="B32" s="206">
+      <c r="A32" s="171" t="s">
+        <v>135</v>
+      </c>
+      <c r="B32" s="172">
         <v>2</v>
       </c>
       <c r="C32">
         <v>115.1</v>
       </c>
-      <c r="D32" s="193"/>
+      <c r="D32" s="168"/>
     </row>
     <row r="33" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="205" t="s">
+      <c r="A33" s="171" t="s">
+        <v>135</v>
+      </c>
+      <c r="B33" s="172">
+        <v>3</v>
+      </c>
+      <c r="C33" s="167"/>
+      <c r="D33" s="168"/>
+    </row>
+    <row r="34" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A34" s="169" t="s">
         <v>136</v>
       </c>
-      <c r="B33" s="206">
-        <v>3</v>
-      </c>
-      <c r="C33" s="192"/>
-      <c r="D33" s="193"/>
-    </row>
-    <row r="34" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A34" s="203" t="s">
-        <v>137</v>
-      </c>
-      <c r="B34" s="204">
+      <c r="B34" s="170">
         <v>1</v>
       </c>
       <c r="C34">
         <v>93.6</v>
       </c>
-      <c r="D34" s="193">
+      <c r="D34" s="168">
         <f>AVERAGE(C34:C36)</f>
         <v>94.05</v>
       </c>
@@ -10517,38 +10565,38 @@
       </c>
     </row>
     <row r="35" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A35" s="203" t="s">
-        <v>137</v>
-      </c>
-      <c r="B35" s="204">
+      <c r="A35" s="169" t="s">
+        <v>136</v>
+      </c>
+      <c r="B35" s="170">
         <v>2</v>
       </c>
       <c r="C35">
         <v>94.5</v>
       </c>
-      <c r="D35" s="193"/>
+      <c r="D35" s="168"/>
     </row>
     <row r="36" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="203" t="s">
+      <c r="A36" s="169" t="s">
+        <v>136</v>
+      </c>
+      <c r="B36" s="170">
+        <v>3</v>
+      </c>
+      <c r="C36" s="167"/>
+      <c r="D36" s="168"/>
+    </row>
+    <row r="37" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A37" s="171" t="s">
         <v>137</v>
       </c>
-      <c r="B36" s="204">
-        <v>3</v>
-      </c>
-      <c r="C36" s="192"/>
-      <c r="D36" s="193"/>
-    </row>
-    <row r="37" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A37" s="205" t="s">
-        <v>138</v>
-      </c>
-      <c r="B37" s="206">
+      <c r="B37" s="172">
         <v>1</v>
       </c>
       <c r="C37">
         <v>71.599999999999994</v>
       </c>
-      <c r="D37" s="193">
+      <c r="D37" s="168">
         <f>AVERAGE(C37:C39)</f>
         <v>71.3</v>
       </c>
@@ -10557,38 +10605,38 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A38" s="205" t="s">
-        <v>138</v>
-      </c>
-      <c r="B38" s="206">
+      <c r="A38" s="171" t="s">
+        <v>137</v>
+      </c>
+      <c r="B38" s="172">
         <v>2</v>
       </c>
       <c r="C38">
         <v>71</v>
       </c>
-      <c r="D38" s="193"/>
+      <c r="D38" s="168"/>
     </row>
     <row r="39" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A39" s="205" t="s">
+      <c r="A39" s="171" t="s">
+        <v>137</v>
+      </c>
+      <c r="B39" s="172">
+        <v>3</v>
+      </c>
+      <c r="C39" s="167"/>
+      <c r="D39" s="168"/>
+    </row>
+    <row r="40" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A40" s="169" t="s">
         <v>138</v>
       </c>
-      <c r="B39" s="206">
-        <v>3</v>
-      </c>
-      <c r="C39" s="192"/>
-      <c r="D39" s="193"/>
-    </row>
-    <row r="40" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="203" t="s">
-        <v>139</v>
-      </c>
-      <c r="B40" s="204">
+      <c r="B40" s="170">
         <v>1</v>
       </c>
       <c r="C40">
         <v>51.8</v>
       </c>
-      <c r="D40" s="193">
+      <c r="D40" s="168">
         <f>AVERAGE(C40:C42)</f>
         <v>50.55</v>
       </c>
@@ -10597,39 +10645,39 @@
       </c>
     </row>
     <row r="41" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A41" s="203" t="s">
-        <v>139</v>
-      </c>
-      <c r="B41" s="204">
+      <c r="A41" s="169" t="s">
+        <v>138</v>
+      </c>
+      <c r="B41" s="170">
         <v>2</v>
       </c>
       <c r="C41">
         <v>49.3</v>
       </c>
-      <c r="D41" s="193"/>
+      <c r="D41" s="168"/>
     </row>
     <row r="42" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A42" s="203" t="s">
+      <c r="A42" s="169" t="s">
+        <v>138</v>
+      </c>
+      <c r="B42" s="170">
+        <v>3</v>
+      </c>
+      <c r="C42" s="167"/>
+      <c r="D42" s="168"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A43" s="171" t="s">
         <v>139</v>
       </c>
-      <c r="B42" s="204">
-        <v>3</v>
-      </c>
-      <c r="C42" s="192"/>
-      <c r="D42" s="193"/>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A43" s="205" t="s">
-        <v>140</v>
-      </c>
-      <c r="B43" s="206">
+      <c r="B43" s="172">
         <v>1</v>
       </c>
       <c r="C43">
         <v>27.8</v>
       </c>
-      <c r="D43" s="193">
-        <f t="shared" ref="D23:D46" si="0">AVERAGE(C43:C45)</f>
+      <c r="D43" s="168">
+        <f t="shared" ref="D43:D46" si="0">AVERAGE(C43:C45)</f>
         <v>27.700000000000003</v>
       </c>
       <c r="E43">
@@ -10637,38 +10685,38 @@
       </c>
     </row>
     <row r="44" spans="1:5" ht="14.65" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A44" s="205" t="s">
-        <v>140</v>
-      </c>
-      <c r="B44" s="206">
+      <c r="A44" s="171" t="s">
+        <v>139</v>
+      </c>
+      <c r="B44" s="172">
         <v>2</v>
       </c>
       <c r="C44">
         <v>27.6</v>
       </c>
-      <c r="D44" s="193"/>
+      <c r="D44" s="168"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A45" s="205" t="s">
-        <v>140</v>
-      </c>
-      <c r="B45" s="206">
+      <c r="A45" s="171" t="s">
+        <v>139</v>
+      </c>
+      <c r="B45" s="172">
         <v>3</v>
       </c>
-      <c r="C45" s="192"/>
-      <c r="D45" s="193"/>
+      <c r="C45" s="167"/>
+      <c r="D45" s="168"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A46" s="205" t="s">
-        <v>140</v>
-      </c>
-      <c r="B46" s="206">
+      <c r="A46" s="171" t="s">
+        <v>139</v>
+      </c>
+      <c r="B46" s="172">
         <v>1</v>
       </c>
       <c r="C46">
         <v>0</v>
       </c>
-      <c r="D46" s="193">
+      <c r="D46" s="168">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -10677,105 +10725,40 @@
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A47" s="205" t="s">
-        <v>140</v>
-      </c>
-      <c r="B47" s="206">
+      <c r="A47" s="171" t="s">
+        <v>139</v>
+      </c>
+      <c r="B47" s="172">
         <v>2</v>
       </c>
       <c r="C47">
         <v>0</v>
       </c>
-      <c r="D47" s="193"/>
+      <c r="D47" s="168"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A48" s="205" t="s">
-        <v>140</v>
-      </c>
-      <c r="B48" s="206">
+      <c r="A48" s="171" t="s">
+        <v>139</v>
+      </c>
+      <c r="B48" s="172">
         <v>3</v>
       </c>
-      <c r="C48" s="192"/>
-      <c r="D48" s="193"/>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B49" s="154"/>
-      <c r="C49" s="154"/>
-      <c r="E49" s="154"/>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B50" s="154"/>
-      <c r="C50" s="154"/>
-      <c r="E50" s="154"/>
-    </row>
-    <row r="51" spans="1:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B51" s="154"/>
-      <c r="C51" s="154"/>
-      <c r="E51" s="154"/>
-    </row>
-    <row r="52" spans="1:6" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A52" s="194" t="s">
-        <v>134</v>
-      </c>
-      <c r="B52" s="195"/>
-      <c r="C52" s="195"/>
-      <c r="D52" s="195"/>
-      <c r="E52" s="195"/>
-      <c r="F52" s="196"/>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A53" s="197"/>
-      <c r="B53" s="198"/>
-      <c r="C53" s="198"/>
-      <c r="D53" s="198"/>
-      <c r="E53" s="198"/>
-      <c r="F53" s="199"/>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A54" s="197"/>
-      <c r="B54" s="198"/>
-      <c r="C54" s="198"/>
-      <c r="D54" s="198"/>
-      <c r="E54" s="198"/>
-      <c r="F54" s="199"/>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A55" s="197"/>
-      <c r="B55" s="198"/>
-      <c r="C55" s="198"/>
-      <c r="D55" s="198"/>
-      <c r="E55" s="198"/>
-      <c r="F55" s="199"/>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A56" s="197"/>
-      <c r="B56" s="198"/>
-      <c r="C56" s="198"/>
-      <c r="D56" s="198"/>
-      <c r="E56" s="198"/>
-      <c r="F56" s="199"/>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A57" s="197"/>
-      <c r="B57" s="198"/>
-      <c r="C57" s="198"/>
-      <c r="D57" s="198"/>
-      <c r="E57" s="198"/>
-      <c r="F57" s="199"/>
-    </row>
-    <row r="58" spans="1:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A58" s="200"/>
-      <c r="B58" s="201"/>
-      <c r="C58" s="201"/>
-      <c r="D58" s="201"/>
-      <c r="E58" s="201"/>
-      <c r="F58" s="202"/>
-    </row>
-    <row r="59" spans="1:6" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
+      <c r="C48" s="167"/>
+      <c r="D48" s="168"/>
+    </row>
+    <row r="49" spans="4:4" s="144" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="D49" s="177"/>
+    </row>
+    <row r="50" spans="4:4" s="144" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="D50" s="177"/>
+    </row>
+    <row r="51" spans="4:4" s="144" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="D51" s="177"/>
+    </row>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="B13:F13"/>
-    <mergeCell ref="A52:F58"/>
+    <mergeCell ref="G2:L8"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="B7:F7"/>
@@ -10865,15 +10848,15 @@
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="144" t="str">
+      <c r="B5" s="209" t="str">
         <f>'Method Comparison'!B5:F5</f>
         <v>This method serves to bringing in-house BNP testing for heart failure assessments</v>
       </c>
-      <c r="C5" s="145"/>
-      <c r="D5" s="145"/>
-      <c r="E5" s="145"/>
-      <c r="F5" s="146"/>
-      <c r="G5" s="147"/>
+      <c r="C5" s="210"/>
+      <c r="D5" s="210"/>
+      <c r="E5" s="210"/>
+      <c r="F5" s="204"/>
+      <c r="G5" s="205"/>
     </row>
     <row r="6" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
@@ -10973,45 +10956,45 @@
       <c r="A18" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="B18" s="148"/>
-      <c r="C18" s="145"/>
-      <c r="D18" s="145"/>
-      <c r="E18" s="145"/>
-      <c r="F18" s="146"/>
-      <c r="G18" s="147"/>
+      <c r="B18" s="211"/>
+      <c r="C18" s="210"/>
+      <c r="D18" s="210"/>
+      <c r="E18" s="210"/>
+      <c r="F18" s="204"/>
+      <c r="G18" s="205"/>
     </row>
     <row r="19" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="B19" s="148"/>
-      <c r="C19" s="145"/>
-      <c r="D19" s="145"/>
-      <c r="E19" s="145"/>
-      <c r="F19" s="146"/>
-      <c r="G19" s="147"/>
+      <c r="B19" s="211"/>
+      <c r="C19" s="210"/>
+      <c r="D19" s="210"/>
+      <c r="E19" s="210"/>
+      <c r="F19" s="204"/>
+      <c r="G19" s="205"/>
     </row>
     <row r="20" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>116</v>
       </c>
-      <c r="B20" s="148"/>
-      <c r="C20" s="145"/>
-      <c r="D20" s="145"/>
-      <c r="E20" s="145"/>
-      <c r="F20" s="146"/>
-      <c r="G20" s="147"/>
+      <c r="B20" s="211"/>
+      <c r="C20" s="210"/>
+      <c r="D20" s="210"/>
+      <c r="E20" s="210"/>
+      <c r="F20" s="204"/>
+      <c r="G20" s="205"/>
     </row>
     <row r="21" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>117</v>
       </c>
-      <c r="B21" s="148"/>
-      <c r="C21" s="145"/>
-      <c r="D21" s="145"/>
-      <c r="E21" s="145"/>
-      <c r="F21" s="146"/>
-      <c r="G21" s="147"/>
+      <c r="B21" s="211"/>
+      <c r="C21" s="210"/>
+      <c r="D21" s="210"/>
+      <c r="E21" s="210"/>
+      <c r="F21" s="204"/>
+      <c r="G21" s="205"/>
     </row>
     <row r="22" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="23" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45"/>

</xml_diff>